<commit_message>
Línea base previa a la reorganización para la copia a la DT
Punto de restauración antes de separar los productos del informe de los
extras (008, 009 y 010 pasan a 9xx_extra_*) y de agregar los scripts de las
tablas que hoy se arman a mano.

Actualiza el insumo SCIAN de junio 2026.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inputs/stps_scian/negociaciones_scian_junio 2026.xlsx
+++ b/inputs/stps_scian/negociaciones_scian_junio 2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://conasamigobmx-my.sharepoint.com/personal/hector_soto_conasami_gob_mx/Documents/Escritorio/CAEL/Informes/Negociación laboral/excels/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://conasamigobmx-my.sharepoint.com/personal/hector_soto_conasami_gob_mx/Documents/Escritorio/CAEL/Informes/Negociación laboral/inputs/stps_scian/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{7470444F-2A19-4484-9B40-FAC8816F42AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60D657C2-242D-40C4-BADA-F5688762B1A7}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{7470444F-2A19-4484-9B40-FAC8816F42AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00CC2842-7956-4D37-9C52-0C61202C557C}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{32627B8B-5DC4-4005-AF49-CA1496A6897D}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
   <si>
     <t>NEGOCIACIONES SALARIALES Y CONTRACTUALES EN LA JURISDICCIÓN FEDERAL POR SECTOR DE ACTIVIDAD ECONÓMICA (SCIAN) MARZO 2024</t>
   </si>
@@ -102,6 +102,9 @@
   </si>
   <si>
     <t>Servicios profesionales, científicos y técnicos</t>
+  </si>
+  <si>
+    <t>Sa</t>
   </si>
 </sst>
 </file>
@@ -586,8 +589,8 @@
       <c r="D4" s="4">
         <v>3.0199999809265137</v>
       </c>
-      <c r="E4" s="3">
-        <v>2</v>
+      <c r="E4" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="F4" s="5">
         <v>0.89999997615814209</v>

</xml_diff>